<commit_message>
Hotfix DCDC auto-Enable applied
</commit_message>
<xml_diff>
--- a/Hardware/Controller/JLC_PCBA_BOM-DALI_EVG_Controller(V0.2).xlsx
+++ b/Hardware/Controller/JLC_PCBA_BOM-DALI_EVG_Controller(V0.2).xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="0" defaultRowHeight="12.75"/>
   <cols>
     <col width="20.2109375" customWidth="1" style="30" min="1" max="2"/>
@@ -1461,22 +1461,18 @@
     <row r="32">
       <c r="A32" s="26" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>15k</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C32" s="19" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
+          <t>Resistor</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="n"/>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>R19, R20</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
@@ -1485,43 +1481,43 @@
         </is>
       </c>
       <c r="F32" s="27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="26" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>Resistor</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>100</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R19, R20</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="F33" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
@@ -1529,10 +1525,14 @@
           <t>Resistor</t>
         </is>
       </c>
-      <c r="C34" s="19" t="n"/>
+      <c r="C34" s="19" t="inlineStr">
+        <is>
+          <t>1.5k</t>
+        </is>
+      </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>R27, R41, R42</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
@@ -1541,13 +1541,13 @@
         </is>
       </c>
       <c r="F34" s="27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="26" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
@@ -1558,7 +1558,7 @@
       <c r="C35" s="19" t="n"/>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>R28</t>
+          <t>R27, R41, R42</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
@@ -1567,13 +1567,13 @@
         </is>
       </c>
       <c r="F35" s="27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="26" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
@@ -1584,7 +1584,7 @@
       <c r="C36" s="19" t="n"/>
       <c r="D36" s="19" t="inlineStr">
         <is>
-          <t>R30</t>
+          <t>R28</t>
         </is>
       </c>
       <c r="E36" s="19" t="inlineStr">
@@ -1599,7 +1599,7 @@
     <row r="37">
       <c r="A37" s="26" t="inlineStr">
         <is>
-          <t>8.2k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="B37" s="19" t="inlineStr">
@@ -1610,7 +1610,7 @@
       <c r="C37" s="19" t="n"/>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>R30</t>
         </is>
       </c>
       <c r="E37" s="19" t="inlineStr">
@@ -1625,7 +1625,7 @@
     <row r="38">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>18k</t>
+          <t>8.2k</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -1636,7 +1636,7 @@
       <c r="C38" s="19" t="n"/>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>R33</t>
+          <t>R32</t>
         </is>
       </c>
       <c r="E38" s="19" t="inlineStr">
@@ -1651,7 +1651,7 @@
     <row r="39">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>33k</t>
+          <t>18k</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
@@ -1662,7 +1662,7 @@
       <c r="C39" s="19" t="n"/>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>R46</t>
+          <t>R33</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
@@ -1677,23 +1677,23 @@
     <row r="40">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>CH32V003F4U6</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>CPU Core:RISC-V CPU Maximum Speed:48MHz Program Storage Size:16KB Number of I/O:18 Applications:-</t>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="C40" s="19" t="n"/>
       <c r="D40" s="19" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R46</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>QFN-20_L3.0-W3.0-P0.40-TL-EP1.7</t>
+          <t>R0603</t>
         </is>
       </c>
       <c r="F40" s="27" t="n">
@@ -1703,23 +1703,23 @@
     <row r="41">
       <c r="A41" s="26" t="inlineStr">
         <is>
-          <t>LMV331IDBVRG4</t>
+          <t>CH32V003F4U6</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>Single General Purpose Low-Voltage Comparator 5-SOT-23</t>
+          <t>CPU Core:RISC-V CPU Maximum Speed:48MHz Program Storage Size:16KB Number of I/O:18 Applications:-</t>
         </is>
       </c>
       <c r="C41" s="19" t="n"/>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>SOT23-5</t>
+          <t>QFN-20_L3.0-W3.0-P0.40-TL-EP1.7</t>
         </is>
       </c>
       <c r="F41" s="27" t="n">
@@ -1729,26 +1729,52 @@
     <row r="42">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>AT24C256C-SSHL-T</t>
+          <t>LMV331IDBVRG4</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>AT24C256C-SSHL-T</t>
+          <t>Single General Purpose Low-Voltage Comparator 5-SOT-23</t>
         </is>
       </c>
       <c r="C42" s="19" t="n"/>
       <c r="D42" s="19" t="inlineStr">
         <is>
+          <t>U2</t>
+        </is>
+      </c>
+      <c r="E42" s="19" t="inlineStr">
+        <is>
+          <t>SOT23-5</t>
+        </is>
+      </c>
+      <c r="F42" s="27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="26" t="inlineStr">
+        <is>
+          <t>AT24C256C-SSHL-T</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="inlineStr">
+        <is>
+          <t>AT24C256C-SSHL-T</t>
+        </is>
+      </c>
+      <c r="C43" s="19" t="n"/>
+      <c r="D43" s="19" t="inlineStr">
+        <is>
           <t>U3</t>
         </is>
       </c>
-      <c r="E42" s="19" t="inlineStr">
+      <c r="E43" s="19" t="inlineStr">
         <is>
           <t>SOIC127P600X265-8N (SOIC-8)</t>
         </is>
       </c>
-      <c r="F42" s="27" t="n">
+      <c r="F43" s="27" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>